<commit_message>
gitignore + soin pokemon + readme
</commit_message>
<xml_diff>
--- a/arenes.xlsx
+++ b/arenes.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="4848" yWindow="3360" windowWidth="17280" windowHeight="8880" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="pokemons" sheetId="1" state="visible" r:id="rId1"/>
@@ -46,8 +46,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -445,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col width="12.6640625" customWidth="1" min="2" max="2"/>
@@ -511,16 +512,16 @@
         <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F2" t="n">
         <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -542,16 +543,16 @@
         <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="F3" t="n">
         <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -573,16 +574,16 @@
         <v>2</v>
       </c>
       <c r="D4" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E4" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
         <v>2</v>
       </c>
       <c r="G4" t="n">
-        <v>2</v>
+        <v>32</v>
       </c>
       <c r="H4" t="n">
         <v>0</v>
@@ -607,7 +608,7 @@
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F5" t="n">
         <v>1</v>
@@ -714,6 +715,9 @@
       <c r="I8" t="n">
         <v>0</v>
       </c>
+    </row>
+    <row r="14">
+      <c r="E14" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>